<commit_message>
update log and testplan
</commit_message>
<xml_diff>
--- a/docs/blazeup/Bug_Tracker.xlsx
+++ b/docs/blazeup/Bug_Tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bug Tracker'!$A$1:$Q$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bug Tracker'!$A$1:$P$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -71,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -79,6 +79,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -529,25 +533,20 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>BE Ticket</t>
+          <t>Reported By</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Reported By</t>
+          <t>Date Opened</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Date Opened</t>
+          <t>Date Closed</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Date Closed</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -559,7 +558,7 @@
           <t>BUG-001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="3" t="n">
         <v>2060122</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -612,19 +611,18 @@
           <t>AssertionError: re-granting must not duplicate active cert</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr"/>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>be_gap — missing idempotency guard</t>
         </is>
@@ -636,7 +634,7 @@
           <t>BUG-002</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="3" t="n">
         <v>2060208</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -689,19 +687,18 @@
           <t>AssertionError: approved deal must stamp rate + rate table version</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr"/>
-      <c r="Q3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>be_gap</t>
         </is>
@@ -713,7 +710,7 @@
           <t>BUG-003</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="3" t="n">
         <v>2060221</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -766,19 +763,18 @@
           <t>CHECK ghost planId (verified absent) -&gt; FAIL (status=201)</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr"/>
-      <c r="Q4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>be_gap — no FK validation</t>
         </is>
@@ -790,9 +786,24 @@
           <t>BUG-004</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="4" t="n">
         <v>2060713</v>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_USERS_013</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Partner Users</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>Major</t>
@@ -810,28 +821,1167 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>FAIL | [2/2] The partner must NOT end up with a duplicate-email user (247ms) -- AssertionError: re-inviting must not duplicate: expected 1 user for qa.auto+gtaylor@mailinator.com, got 2 — BE creates a</t>
+          <t>Inviting a duplicate email creates a second user</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Reject (409) or idempotent — no duplicate user</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Returns 201; two users share one login</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>AssertionError: re-inviting must not duplicate user</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>QA</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
           <t>2026-07-20</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>auto-added by AI triage</t>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>be_gap — no duplicate-email guard</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BUG-005</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>2061003</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PARTNER_API_AUTH_ACCESS_CONTROL_003</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>AUTH_ACCESS_CONTROL</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>cross-partner access - a partner cannot read another's deal.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>404 (preferred, hides existence) or 403 for cross-partner access</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Returns 400 (mislabels a valid request as malformed); isolation holds (no data leak)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>FAIL | [1/1] Partner B requests partner A's deal → refused, no leak (333ms) -- AssertionError: cross-partner access should be 404 (preferred) or 403, got 400 — BE returns 400 (a valid request, not a bad one); confirm with BE</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>AI Triage</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>be_gap — wrong status code for authz; confirm with BE (should be 404)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BUG-006</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>2060231</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>PARTNER_API_DEAL_REGISTRATION_PIPELINE_031</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>DEAL_REGISTRATION_PIPELINE</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>GET deal by a well-formed but non-existent id returns 400 instead of 404</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>404 Not Found for a well-formed but non-existent deal id</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>400 Bad Request with message "Deal 000000000000000000000000 not found" (status contradicts message)</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>test_partner_api_deal_registration_pipeline_031 [1/2]: expected 404, got 400, msg="Deal 000000000000000000000000 not found"</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>QA (review)</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>REST-hygiene: malformed id -&gt; 400 is correct; a well-formed absent id should be 404. be_gap, excluded from merge gate. Confirm with BE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BUG-007</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>2060232</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>PARTNER_API_DEAL_REGISTRATION_PIPELINE_032</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>DEAL_REGISTRATION_PIPELINE</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>lose deal on a well-formed but non-existent id returns 400 instead of 404</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>404 Not Found for a well-formed but non-existent deal id</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>400 Bad Request with message "Deal 000000000000000000000000 not found" (status contradicts message)</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>test_partner_api_deal_registration_pipeline_032 [2/3]: expected 404, got 400, msg="Deal 000000000000000000000000 not found"</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>QA (review)</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Same root cause as BUG-006 (get-by-id). Ghost id -&gt; should be 404. Illegal-transition (400) and malformed (400) cases are correct. be_gap, excluded from merge gate. Confirm with BE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BUG-008</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>2060228</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>PARTNER_API_DEAL_REGISTRATION_PIPELINE_028</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>DEAL_REGISTRATION_PIPELINE</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>approve deal on a well-formed but non-existent id returns 400 instead of 404</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>404 Not Found for a well-formed but non-existent deal id</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>400 Bad Request with message "Deal 000000000000000000000000 not found" (status contradicts message)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>test_partner_api_deal_registration_pipeline_028 [1/3]: expected 404, got 400, msg="Deal 000000000000000000000000 not found"</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>QA (review)</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Same root cause as BUG-006/007 (ghost id -&gt; should be 404). Malformed (400) and illegal-transition (400) cases are correct. be_gap, excluded from merge gate. Confirm with BE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BUG-009</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>2060229</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>PARTNER_API_DEAL_REGISTRATION_PIPELINE_029</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>DEAL_REGISTRATION_PIPELINE</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>resolve-conflict on a well-formed but non-existent id returns 400 instead of 404</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>404 Not Found for a well-formed but non-existent deal id</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>400 Bad Request with message "Deal 000000000000000000000000 not found" (status contradicts message)</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>test_partner_api_deal_registration_pipeline_029 [6/6]: expected 404, got 400, msg="Deal 000000000000000000000000 not found"</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>QA (review)</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Same root cause as BUG-006/007/008 (ghost id -&gt; should be 404). Validation/format/state cases (400) are correct. be_gap, excluded from merge gate. Confirm with BE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BUG-010</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>2060230</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>PARTNER_API_DEAL_REGISTRATION_PIPELINE_030</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>DEAL_REGISTRATION_PIPELINE</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>extend-protection on a well-formed but non-existent id returns 400 instead of 404</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>404 Not Found for a well-formed but non-existent deal id</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>400 Bad Request with message "Deal 000000000000000000000000 not found" (status contradicts message)</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>test_partner_api_deal_registration_pipeline_030 [8/8]: expected 404, got 400, msg="Deal 000000000000000000000000 not found"</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>QA (review)</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Same root cause as BUG-006/007/008/009 (ghost id -&gt; should be 404). Body-validation/boundary/format/malformed cases (400) are correct. be_gap, excluded from merge gate. Confirm with BE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BUG-011</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>2061111</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PARTNER_API_DEAL_APPROVAL_QUEUE_011</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>DEAL_APPROVAL_QUEUE</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>reject deal on a well-formed but non-existent id returns 400 instead of 404</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>404 Not Found for a well-formed but non-existent deal id</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>400 Bad Request with message "Deal 000000000000000000000000 not found" (status contradicts message)</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>test_partner_api_deal_approval_queue_011 [1/3]: expected 404, got 400, msg="Deal 000000000000000000000000 not found"</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>QA (review)</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Same root cause as BUG-006..010 (ghost path id -&gt; should be 404). Malformed (400) and illegal-transition (400) cases are correct. be_gap, excluded from merge gate. Confirm with BE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BUG-012</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>2060113</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_ACCOUNT_MANAGEMENT_013</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>PARTNER_ACCOUNT_MANAGEMENT</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>approve partner: well-formed but non-existent partner id returns 400 instead of 404</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>404 Not Found for a well-formed but non-existent partner id</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>400 Bad Request with message "Partner 000000000000000000000000 not found" (status contradicts message)</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>test_partner_api_partner_account_management_013 [1/3]: expected 404, got 400, msg="Partner 000000000000000000000000 not found"</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>QA (review)</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Same root cause as BUG-006..011 (ghost path id -&gt; should be 404), now on partner-id endpoints. Other cases (validation/format/transition, all 400) are correct. be_gap, excluded from merge gate. Confirm with BE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BUG-013</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>2060114</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_ACCOUNT_MANAGEMENT_014</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>PARTNER_ACCOUNT_MANAGEMENT</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>deactivate partner: well-formed but non-existent partner id returns 400 instead of 404</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>404 Not Found for a well-formed but non-existent partner id</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>400 Bad Request with message "Partner 000000000000000000000000 not found" (status contradicts message)</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>test_partner_api_partner_account_management_014 [1/3]: expected 404, got 400, msg="Partner 000000000000000000000000 not found"</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>QA (review)</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Same root cause as BUG-006..011 (ghost path id -&gt; should be 404), now on partner-id endpoints. Other cases (validation/format/transition, all 400) are correct. be_gap, excluded from merge gate. Confirm with BE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BUG-014</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>2060115</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_ACCOUNT_MANAGEMENT_015</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>PARTNER_ACCOUNT_MANAGEMENT</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>change-tier partner: well-formed but non-existent partner id returns 400 instead of 404</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>404 Not Found for a well-formed but non-existent partner id</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>400 Bad Request with message "Partner 000000000000000000000000 not found" (status contradicts message)</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>test_partner_api_partner_account_management_015 [6/6]: expected 404, got 400, msg="Partner 000000000000000000000000 not found"</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>QA (review)</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Same root cause as BUG-006..011 (ghost path id -&gt; should be 404), now on partner-id endpoints. Other cases (validation/format/transition, all 400) are correct. be_gap, excluded from merge gate. Confirm with BE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BUG-015</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>2060120</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_ACCOUNT_MANAGEMENT_020</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>PARTNER_ACCOUNT_MANAGEMENT</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>grant-certification on a well-formed but non-existent userId returns 400 instead of 404</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>404 Not Found for a well-formed but non-existent userId</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>400 Bad Request with message "User 000000000000000000000000 not found" (status contradicts message)</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>test_partner_api_partner_account_management_020 [4/4]: expected 404, got 400, msg="User 000000000000000000000000 not found"</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>QA (review)</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Same root cause as BUG-006..014 (ghost path id -&gt; should be 404), on partner-users/{userId} endpoint. Validation/format cases (400) are correct. be_gap, excluded from merge gate. Confirm with BE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BUG-016</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>2060714</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>PARTNER_API_PARTNER_USERS_014</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>PARTNER_USERS</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>reset-password on a well-formed but non-existent userId returns 400 instead of 404</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>404 Not Found for a well-formed but non-existent userId</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>400 Bad Request with message "User 000000000000000000000000 not found" (status contradicts message)</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>test_partner_api_partner_users_014 [1/2]: expected 404, got 400, msg="User 000000000000000000000000 not found"</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>QA (review)</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Same root cause as BUG-006..015 (ghost path id -&gt; should be 404), on partner-users/{userId}/reset-password. Malformed (400) is correct. be_gap, excluded from merge gate. Confirm with BE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BUG-017</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>2060414</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>PARTNER_API_TERRITORIES_014</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>TERRITORIES</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>get-territory-by-id on a well-formed but non-existent id returns 400 instead of 404</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>404 Not Found for a well-formed but non-existent / already-removed territory id</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>400 Bad Request with message "Territory ... not found" (status contradicts message)</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>test_partner_api_territories_014 [1/2]: expected 404, got 400, msg="Territory 000000000000000000000000 not found"</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>QA (review)</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Same root cause as BUG-006..016 (ghost path id -&gt; should be 404), on territories endpoints. Malformed (400) is correct. be_gap, excluded from merge gate. Confirm with BE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BUG-018</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>2060415</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>PARTNER_API_TERRITORIES_015</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>TERRITORIES</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>delete territory on a non-existent / already-removed id returns 400 instead of 404</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>404 Not Found for a well-formed but non-existent / already-removed territory id</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>400 Bad Request with message "Territory ... not found" (status contradicts message)</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>test_partner_api_territories_015 [1/3] + [3/3]: expected 404, got 400 (ghost id AND already-removed), msg="Territory ... not found"</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>QA (review)</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Same root cause as BUG-006..016 (ghost path id -&gt; should be 404), on territories endpoints. Malformed (400) is correct. be_gap, excluded from merge gate. Confirm with BE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BUG-019</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>2060512</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>PARTNER_API_CERTIFICATIONS_SA_012</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>CERTIFICATIONS_SA</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>revoke-certification not-found targets (ghost user / cert-not-held / already-revoked) return 400 instead of 404</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>404 Not Found when the revoke target (user or active cert) does not exist</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>400 Bad Request with a "not found" message (User ... not found / Active ... certification not found)</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>test_partner_api_certifications_sa_012: cases 2,3,5 expected 404, got 400 (msg contains not found)</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>QA (review)</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Same root cause as BUG-006..018 (not-found -&gt; should be 404). Missing-reason (400) and malformed-id (400) are correct. be_gap, excluded from merge gate. Confirm with BE.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q1"/>
+  <autoFilter ref="A1:P1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
verify and modify 12060507
</commit_message>
<xml_diff>
--- a/docs/blazeup/Bug_Tracker.xlsx
+++ b/docs/blazeup/Bug_Tracker.xlsx
@@ -2512,7 +2512,7 @@
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>CLOSE</t>
         </is>
       </c>
       <c r="I30" s="7" t="inlineStr">
@@ -2545,10 +2545,14 @@
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="O30" s="7" t="n"/>
+      <c r="O30" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
       <c r="P30" s="7" t="inlineStr">
         <is>
-          <t>Root cause = contract drift: a plan-slug "pro-v1" (string) is used where the API expects a Mongo _id (24-hex), so deal-list id validation fails. CONSISTENT, not intermittent (updated 2026-08-05): earlier "lucky PASS" runs were a TEST race - the assertion ran before the async deal-list error painted; the test now waits for the fetch to settle and fails deterministically. UI test 12060507 renders fine (shell/filters/headers OK); this step reflects the BE defect. Fix BE so deal-list never returns Invalid id: pro-v1.</t>
+          <t>FIXED — re-verified 2026-08-10: PARTNER_UI_SA_PARTNER_MODULE_007 now PASSES (15.3s, log: 'CHECK deals load -&gt; OK (no server error)'). The deal-list fetch no longer returns "Invalid id: 'pro-v1'". be_gap marker removed from the test and the registry re-synced, so this TC is back inside the merge gate. | Root cause = contract drift: a plan-slug "pro-v1" (string) is used where the API expects a Mongo _id (24-hex), so deal-list id validation fails. CONSISTENT, not intermittent (updated 2026-08-05): earlier "lucky PASS" runs were a TEST race - the assertion ran before the async deal-list error painted; the test now waits for the fetch to settle and fails deterministically. UI test 12060507 renders fine (shell/filters/headers OK); this step reflects the BE defect. Fix BE so deal-list never returns Invalid id: pro-v1.</t>
         </is>
       </c>
     </row>

</xml_diff>